<commit_message>
add new progress for HW9
</commit_message>
<xml_diff>
--- a/HW9/result/HW9.xlsx
+++ b/HW9/result/HW9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T00229\Documents\GitHub\DADS7102\HW9\result\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nuna\Documents\GitHub\DADS7102\HW9\result\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65717451-0EFB-43D3-BB6E-D2828BC82F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00509A89-372F-409A-BF9E-F95F96C3E93E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7DD5DE49-5239-4E35-A7A7-CFC750C4AB3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7DD5DE49-5239-4E35-A7A7-CFC750C4AB3D}"/>
   </bookViews>
   <sheets>
     <sheet name="HW9" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,8 @@
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">'HW9'!$AD$9</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">'HW9'!$AD$10:$AD$21</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">'HW9'!$AD$10:$AD$21</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">'HW9'!$AD$9</definedName>
     <definedName name="solver_lhs3" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
     <definedName name="solver_lhs4" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
     <definedName name="solver_lhs5" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
@@ -38,13 +38,13 @@
     <definedName name="solver_opt" localSheetId="0" hidden="1">'HW9'!$AD$8</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel3" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_rel4" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel5" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_rhs1" localSheetId="0" hidden="1">'HW9'!$AF$9</definedName>
-    <definedName name="solver_rhs2" localSheetId="0" hidden="1">'HW9'!$AF$10:$AF$21</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">'HW9'!$AF$10:$AF$21</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">'HW9'!$AF$9</definedName>
     <definedName name="solver_rhs3" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
     <definedName name="solver_rhs4" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
     <definedName name="solver_rhs5" localSheetId="0" hidden="1">'HW9'!#REF!</definedName>
@@ -243,7 +243,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -261,7 +261,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -298,6 +298,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -492,9 +498,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
@@ -504,9 +510,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -514,15 +517,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -540,24 +537,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -902,80 +899,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D1" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="H1" t="s">
+      <c r="F1" s="7"/>
+      <c r="H1" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="I1">
+      <c r="I1" s="35">
         <v>150</v>
       </c>
-      <c r="J1">
-        <v>150</v>
-      </c>
-      <c r="K1">
+      <c r="J1" s="35">
+        <v>230</v>
+      </c>
+      <c r="K1" s="35">
         <v>260</v>
       </c>
-      <c r="L1">
+      <c r="L1" s="35">
         <v>238</v>
       </c>
-      <c r="M1">
+      <c r="M1" s="35">
         <v>210</v>
       </c>
-      <c r="N1">
+      <c r="N1" s="35">
         <v>-170</v>
       </c>
-      <c r="O1">
+      <c r="O1" s="35">
         <v>-150</v>
       </c>
-      <c r="P1">
+      <c r="P1" s="35">
         <v>-36</v>
       </c>
-      <c r="Q1">
+      <c r="Q1" s="35">
         <v>-10</v>
       </c>
-      <c r="R1">
+      <c r="R1" s="35">
         <v>238</v>
       </c>
-      <c r="S1">
+      <c r="S1" s="35">
         <v>210</v>
       </c>
-      <c r="T1">
+      <c r="T1" s="35">
         <v>-170</v>
       </c>
-      <c r="U1">
+      <c r="U1" s="35">
         <v>-150</v>
       </c>
-      <c r="V1">
+      <c r="V1" s="35">
         <v>-36</v>
       </c>
-      <c r="W1">
+      <c r="W1" s="35">
         <v>-10</v>
       </c>
-      <c r="X1">
+      <c r="X1" s="35">
         <v>238</v>
       </c>
-      <c r="Y1">
+      <c r="Y1" s="35">
         <v>210</v>
       </c>
-      <c r="Z1">
+      <c r="Z1" s="35">
         <v>-170</v>
       </c>
-      <c r="AA1">
+      <c r="AA1" s="35">
         <v>-150</v>
       </c>
-      <c r="AB1">
+      <c r="AB1" s="35">
         <v>-36</v>
       </c>
-      <c r="AC1">
+      <c r="AC1" s="35">
         <v>-10</v>
       </c>
     </row>
@@ -992,89 +989,89 @@
       <c r="D2">
         <v>20</v>
       </c>
-      <c r="F2" s="8"/>
+      <c r="F2" s="7"/>
       <c r="H2" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="37">
-        <v>1</v>
-      </c>
-      <c r="J2" s="37">
-        <v>1</v>
-      </c>
-      <c r="K2" s="37">
-        <v>1</v>
-      </c>
-      <c r="L2" s="37">
-        <f>1/3</f>
+      <c r="I2" s="30">
+        <v>1</v>
+      </c>
+      <c r="J2" s="30">
+        <v>1</v>
+      </c>
+      <c r="K2" s="30">
+        <v>1</v>
+      </c>
+      <c r="L2" s="30">
+        <f t="shared" ref="L2:AC2" si="0">1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="M2" s="37">
-        <f>1/3</f>
+      <c r="M2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="N2" s="37">
-        <f>1/3</f>
+      <c r="N2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="O2" s="37">
-        <f>1/3</f>
+      <c r="O2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="P2" s="37">
-        <f>1/3</f>
+      <c r="P2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="Q2" s="37">
-        <f>1/3</f>
+      <c r="Q2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="R2" s="37">
-        <f>1/3</f>
+      <c r="R2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="S2" s="37">
-        <f>1/3</f>
+      <c r="S2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="T2" s="37">
-        <f>1/3</f>
+      <c r="T2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="U2" s="37">
-        <f>1/3</f>
+      <c r="U2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="V2" s="37">
-        <f>1/3</f>
+      <c r="V2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="W2" s="37">
-        <f>1/3</f>
+      <c r="W2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="X2" s="37">
-        <f>1/3</f>
+      <c r="X2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="Y2" s="37">
-        <f>1/3</f>
+      <c r="Y2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="Z2" s="37">
-        <f>1/3</f>
+      <c r="Z2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="AA2" s="37">
-        <f>1/3</f>
+      <c r="AA2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="AB2" s="37">
-        <f>1/3</f>
+      <c r="AB2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="AC2" s="37">
-        <f>1/3</f>
+      <c r="AC2" s="30">
+        <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
     </row>
@@ -1091,7 +1088,7 @@
       <c r="D3">
         <v>260</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="7"/>
       <c r="H3" t="s">
         <v>45</v>
       </c>
@@ -1105,10 +1102,10 @@
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="N3">
         <v>0.9</v>
@@ -1141,10 +1138,10 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Y3">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Z3">
         <v>1.1000000000000001</v>
@@ -1169,95 +1166,95 @@
       <c r="C4">
         <v>240</v>
       </c>
-      <c r="D4" s="36">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8"/>
+      <c r="D4" s="29">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7"/>
       <c r="H4" t="s">
         <v>43</v>
       </c>
       <c r="I4">
-        <f>I1*I3</f>
+        <f t="shared" ref="I4:AC4" si="1">I1*I3</f>
         <v>150</v>
       </c>
       <c r="J4">
-        <f>J1*J3</f>
-        <v>150</v>
+        <f t="shared" si="1"/>
+        <v>230</v>
       </c>
       <c r="K4">
-        <f>K1*K3</f>
+        <f t="shared" si="1"/>
         <v>260</v>
       </c>
       <c r="L4">
-        <f>L1*L3</f>
+        <f t="shared" si="1"/>
+        <v>214.20000000000002</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="1"/>
+        <v>189</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="1"/>
+        <v>-153</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="1"/>
+        <v>-135</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="1"/>
+        <v>-36</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="1"/>
+        <v>-10</v>
+      </c>
+      <c r="R4">
+        <f t="shared" si="1"/>
         <v>238</v>
       </c>
-      <c r="M4">
-        <f>M1*M3</f>
+      <c r="S4">
+        <f t="shared" si="1"/>
         <v>210</v>
       </c>
-      <c r="N4">
-        <f>N1*N3</f>
-        <v>-153</v>
-      </c>
-      <c r="O4">
-        <f>O1*O3</f>
-        <v>-135</v>
-      </c>
-      <c r="P4">
-        <f>P1*P3</f>
+      <c r="T4">
+        <f t="shared" si="1"/>
+        <v>-170</v>
+      </c>
+      <c r="U4">
+        <f t="shared" si="1"/>
+        <v>-150</v>
+      </c>
+      <c r="V4">
+        <f t="shared" si="1"/>
         <v>-36</v>
       </c>
-      <c r="Q4">
-        <f>Q1*Q3</f>
+      <c r="W4">
+        <f t="shared" si="1"/>
         <v>-10</v>
       </c>
-      <c r="R4">
-        <f>R1*R3</f>
-        <v>238</v>
-      </c>
-      <c r="S4">
-        <f>S1*S3</f>
-        <v>210</v>
-      </c>
-      <c r="T4">
-        <f>T1*T3</f>
-        <v>-170</v>
-      </c>
-      <c r="U4">
-        <f>U1*U3</f>
-        <v>-150</v>
-      </c>
-      <c r="V4">
-        <f>V1*V3</f>
+      <c r="X4">
+        <f t="shared" si="1"/>
+        <v>261.8</v>
+      </c>
+      <c r="Y4">
+        <f t="shared" si="1"/>
+        <v>231.00000000000003</v>
+      </c>
+      <c r="Z4">
+        <f t="shared" si="1"/>
+        <v>-187.00000000000003</v>
+      </c>
+      <c r="AA4">
+        <f t="shared" si="1"/>
+        <v>-165</v>
+      </c>
+      <c r="AB4">
+        <f t="shared" si="1"/>
         <v>-36</v>
       </c>
-      <c r="W4">
-        <f>W1*W3</f>
-        <v>-10</v>
-      </c>
-      <c r="X4">
-        <f>X1*X3</f>
-        <v>238</v>
-      </c>
-      <c r="Y4">
-        <f>Y1*Y3</f>
-        <v>210</v>
-      </c>
-      <c r="Z4">
-        <f>Z1*Z3</f>
-        <v>-187.00000000000003</v>
-      </c>
-      <c r="AA4">
-        <f>AA1*AA3</f>
-        <v>-165</v>
-      </c>
-      <c r="AB4">
-        <f>AB1*AB3</f>
-        <v>-36</v>
-      </c>
       <c r="AC4">
-        <f>AC1*AC3</f>
+        <f t="shared" si="1"/>
         <v>-10</v>
       </c>
     </row>
@@ -1271,10 +1268,10 @@
       <c r="C5">
         <v>210</v>
       </c>
-      <c r="D5" s="36">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8"/>
+      <c r="D5" s="29">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
@@ -1283,68 +1280,68 @@
       <c r="E6" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="I6" s="35" t="s">
+      <c r="F6" s="7"/>
+      <c r="I6" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="34" t="s">
+      <c r="J6" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="34" t="s">
+      <c r="K6" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="L6" s="35" t="s">
+      <c r="L6" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M6" s="34" t="s">
+      <c r="M6" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="N6" s="34" t="s">
+      <c r="N6" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="34" t="s">
+      <c r="O6" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="P6" s="34" t="s">
+      <c r="P6" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="Q6" s="33" t="s">
+      <c r="Q6" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="R6" s="35" t="s">
+      <c r="R6" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="S6" s="34" t="s">
+      <c r="S6" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="T6" s="34" t="s">
+      <c r="T6" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="U6" s="34" t="s">
+      <c r="U6" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="V6" s="34" t="s">
+      <c r="V6" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="33" t="s">
+      <c r="W6" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="X6" s="32" t="s">
+      <c r="X6" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="Y6" s="32" t="s">
+      <c r="Y6" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="Z6" s="32" t="s">
+      <c r="Z6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="AA6" s="32" t="s">
+      <c r="AA6" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="AB6" s="32" t="s">
+      <c r="AB6" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="AC6" s="32" t="s">
+      <c r="AC6" s="28" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1364,71 +1361,71 @@
       <c r="E7">
         <v>10</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="H7" s="28" t="s">
+      <c r="F7" s="7"/>
+      <c r="H7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="31">
-        <v>88.888888888888943</v>
-      </c>
-      <c r="J7" s="31">
-        <v>138.38383838383834</v>
-      </c>
-      <c r="K7" s="31">
+      <c r="I7" s="27">
+        <v>138.38383838383842</v>
+      </c>
+      <c r="J7" s="27">
+        <v>88.888888888888886</v>
+      </c>
+      <c r="K7" s="27">
         <v>272.72727272727269</v>
       </c>
-      <c r="L7" s="31">
-        <v>0</v>
-      </c>
-      <c r="M7" s="31">
-        <v>0</v>
-      </c>
-      <c r="N7" s="31">
-        <v>44.444444444444429</v>
-      </c>
-      <c r="O7" s="31">
-        <v>216.66666666666663</v>
-      </c>
-      <c r="P7" s="31">
+      <c r="L7" s="27">
+        <v>0</v>
+      </c>
+      <c r="M7" s="27">
+        <v>0</v>
+      </c>
+      <c r="N7" s="27">
+        <v>180.55555555555546</v>
+      </c>
+      <c r="O7" s="27">
+        <v>53.333333333333371</v>
+      </c>
+      <c r="P7" s="27">
         <v>5999.9999999999991</v>
       </c>
-      <c r="Q7" s="31">
-        <v>0</v>
-      </c>
-      <c r="R7" s="31">
-        <v>0</v>
-      </c>
-      <c r="S7" s="31">
-        <v>0</v>
-      </c>
-      <c r="T7" s="31">
-        <v>22.222222222222086</v>
-      </c>
-      <c r="U7" s="31">
-        <v>175.15151515151504</v>
-      </c>
-      <c r="V7" s="31">
+      <c r="Q7" s="27">
+        <v>0</v>
+      </c>
+      <c r="R7" s="27">
+        <v>0</v>
+      </c>
+      <c r="S7" s="27">
+        <v>0</v>
+      </c>
+      <c r="T7" s="27">
+        <v>145.95959595959567</v>
+      </c>
+      <c r="U7" s="27">
+        <v>26.666666666666664</v>
+      </c>
+      <c r="V7" s="27">
         <v>5454.545454545455</v>
       </c>
-      <c r="W7" s="31">
-        <v>0</v>
-      </c>
-      <c r="X7" s="30">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="30">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="30">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="30">
-        <v>133.63636363636354</v>
-      </c>
-      <c r="AB7" s="30">
+      <c r="W7" s="27">
+        <v>0</v>
+      </c>
+      <c r="X7" s="27">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="27">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="27">
+        <v>111.36363636363626</v>
+      </c>
+      <c r="AA7" s="27">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="27">
         <v>4909.090909090909</v>
       </c>
-      <c r="AC7" s="30">
+      <c r="AC7" s="27">
         <v>0</v>
       </c>
     </row>
@@ -1452,97 +1449,97 @@
         <f>D2*E7-D3</f>
         <v>-60</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="H8" s="28" t="s">
+      <c r="F8" s="7"/>
+      <c r="H8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="16">
-        <f>I1*I2</f>
+      <c r="I8" s="25">
+        <f>I4*I2</f>
         <v>150</v>
       </c>
-      <c r="J8" s="15">
-        <f>J1*J2</f>
-        <v>150</v>
-      </c>
-      <c r="K8" s="15">
-        <f>K1*K2</f>
+      <c r="J8" s="25">
+        <f t="shared" ref="J8:AC8" si="2">J4*J2</f>
+        <v>230</v>
+      </c>
+      <c r="K8" s="25">
+        <f t="shared" si="2"/>
         <v>260</v>
       </c>
-      <c r="L8" s="16">
-        <f>L1*L2</f>
+      <c r="L8" s="25">
+        <f t="shared" si="2"/>
+        <v>71.400000000000006</v>
+      </c>
+      <c r="M8" s="25">
+        <f t="shared" si="2"/>
+        <v>63</v>
+      </c>
+      <c r="N8" s="25">
+        <f t="shared" si="2"/>
+        <v>-51</v>
+      </c>
+      <c r="O8" s="25">
+        <f t="shared" si="2"/>
+        <v>-45</v>
+      </c>
+      <c r="P8" s="25">
+        <f t="shared" si="2"/>
+        <v>-12</v>
+      </c>
+      <c r="Q8" s="25">
+        <f t="shared" si="2"/>
+        <v>-3.333333333333333</v>
+      </c>
+      <c r="R8" s="25">
+        <f t="shared" si="2"/>
         <v>79.333333333333329</v>
       </c>
-      <c r="M8" s="15">
-        <f>M1*M2</f>
+      <c r="S8" s="25">
+        <f t="shared" si="2"/>
         <v>70</v>
       </c>
-      <c r="N8" s="15">
-        <f>N1*N2</f>
+      <c r="T8" s="25">
+        <f>T4*T2</f>
         <v>-56.666666666666664</v>
       </c>
-      <c r="O8" s="15">
-        <f>O1*O2</f>
+      <c r="U8" s="25">
+        <f t="shared" si="2"/>
         <v>-50</v>
       </c>
-      <c r="P8" s="15">
-        <f>P1*P2</f>
+      <c r="V8" s="25">
+        <f t="shared" si="2"/>
         <v>-12</v>
       </c>
-      <c r="Q8" s="14">
-        <f>Q1*Q2</f>
+      <c r="W8" s="25">
+        <f t="shared" si="2"/>
         <v>-3.333333333333333</v>
       </c>
-      <c r="R8" s="16">
-        <f>R1*R2</f>
-        <v>79.333333333333329</v>
-      </c>
-      <c r="S8" s="15">
-        <f>S1*S2</f>
-        <v>70</v>
-      </c>
-      <c r="T8" s="15">
-        <f>T1*T2</f>
-        <v>-56.666666666666664</v>
-      </c>
-      <c r="U8" s="15">
-        <f>U1*U2</f>
-        <v>-50</v>
-      </c>
-      <c r="V8" s="15">
-        <f>V1*V2</f>
+      <c r="X8" s="25">
+        <f t="shared" si="2"/>
+        <v>87.266666666666666</v>
+      </c>
+      <c r="Y8" s="25">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+      <c r="Z8" s="25">
+        <f t="shared" si="2"/>
+        <v>-62.333333333333343</v>
+      </c>
+      <c r="AA8" s="25">
+        <f t="shared" si="2"/>
+        <v>-55</v>
+      </c>
+      <c r="AB8" s="25">
+        <f t="shared" si="2"/>
         <v>-12</v>
       </c>
-      <c r="W8" s="14">
-        <f>W1*W2</f>
+      <c r="AC8" s="25">
+        <f t="shared" si="2"/>
         <v>-3.333333333333333</v>
       </c>
-      <c r="X8" s="28">
-        <f>X1*X2</f>
-        <v>79.333333333333329</v>
-      </c>
-      <c r="Y8" s="28">
-        <f>Y1*Y2</f>
-        <v>70</v>
-      </c>
-      <c r="Z8" s="28">
-        <f>Z1*Z2</f>
-        <v>-56.666666666666664</v>
-      </c>
-      <c r="AA8" s="28">
-        <f>AA1*AA2</f>
-        <v>-50</v>
-      </c>
-      <c r="AB8" s="28">
-        <f>AB1*AB2</f>
-        <v>-12</v>
-      </c>
-      <c r="AC8" s="28">
-        <f>AC1*AC2</f>
-        <v>-3.333333333333333</v>
-      </c>
-      <c r="AD8" s="29">
-        <f>SUMPRODUCT(I8:AC8,$I$7:$AC$7)</f>
-        <v>-121414.14141414137</v>
+      <c r="AD8" s="26">
+        <f t="shared" ref="AD8:AD21" si="3">SUMPRODUCT(I8:AC8,$I$7:$AC$7)</f>
+        <v>-112406.90235690231</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
@@ -1561,124 +1558,124 @@
       <c r="E9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="H9" s="28" t="s">
+      <c r="F9" s="7"/>
+      <c r="H9" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="26">
-        <v>1</v>
-      </c>
-      <c r="J9" s="25">
-        <v>1</v>
-      </c>
-      <c r="K9" s="25">
-        <v>1</v>
-      </c>
-      <c r="L9" s="26"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
-      <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="27"/>
-      <c r="T9" s="25"/>
-      <c r="U9" s="25"/>
-      <c r="V9" s="25"/>
-      <c r="W9" s="24"/>
-      <c r="X9" s="26"/>
-      <c r="Y9" s="25"/>
-      <c r="Z9" s="25"/>
-      <c r="AA9" s="25"/>
-      <c r="AB9" s="25"/>
-      <c r="AC9" s="24"/>
+      <c r="I9" s="23">
+        <v>1</v>
+      </c>
+      <c r="J9" s="22">
+        <v>1</v>
+      </c>
+      <c r="K9" s="22">
+        <v>1</v>
+      </c>
+      <c r="L9" s="23"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="23"/>
+      <c r="S9" s="24"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="21"/>
+      <c r="X9" s="23"/>
+      <c r="Y9" s="22"/>
+      <c r="Z9" s="22"/>
+      <c r="AA9" s="22"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="21"/>
       <c r="AD9" s="3">
-        <f>SUMPRODUCT(I9:AC9,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>500</v>
       </c>
-      <c r="AE9" s="19" t="s">
+      <c r="AE9" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="AF9" s="18">
+      <c r="AF9" s="15">
         <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F10" s="8"/>
-      <c r="G10" s="17" t="s">
+      <c r="F10" s="7"/>
+      <c r="G10" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="14">
         <f>1.1*2.5</f>
         <v>2.75</v>
       </c>
-      <c r="J10" s="15">
-        <v>0</v>
-      </c>
-      <c r="K10" s="14">
-        <v>0</v>
-      </c>
-      <c r="L10" s="16">
-        <v>1</v>
-      </c>
-      <c r="M10" s="15">
-        <v>0</v>
-      </c>
-      <c r="N10" s="15">
+      <c r="J10" s="13">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <v>0</v>
+      </c>
+      <c r="L10" s="14">
+        <v>1</v>
+      </c>
+      <c r="M10" s="13">
+        <v>0</v>
+      </c>
+      <c r="N10" s="13">
         <v>-1</v>
       </c>
-      <c r="O10" s="15">
-        <v>0</v>
-      </c>
-      <c r="P10" s="15">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="14">
-        <v>0</v>
-      </c>
-      <c r="R10" s="16"/>
-      <c r="S10" s="23"/>
-      <c r="T10" s="15"/>
-      <c r="U10" s="15"/>
-      <c r="V10" s="15"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="15"/>
-      <c r="Z10" s="15"/>
-      <c r="AA10" s="15"/>
-      <c r="AB10" s="15"/>
-      <c r="AC10" s="14"/>
+      <c r="O10" s="13">
+        <v>0</v>
+      </c>
+      <c r="P10" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="12">
+        <v>0</v>
+      </c>
+      <c r="R10" s="14"/>
+      <c r="S10" s="20"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="14"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="12"/>
       <c r="AD10" s="3">
-        <f>SUMPRODUCT(I10:AC10,$I$7:$AC$7)</f>
-        <v>200.00000000000017</v>
-      </c>
-      <c r="AE10" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF10" s="21">
+        <f t="shared" si="3"/>
+        <v>200.0000000000002</v>
+      </c>
+      <c r="AE10" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="18">
         <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F11" s="8"/>
-      <c r="G11" s="13"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="33"/>
       <c r="H11" t="s">
         <v>3</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="11">
         <v>0</v>
       </c>
       <c r="J11">
         <f>1.1*3</f>
         <v>3.3000000000000003</v>
       </c>
-      <c r="K11" s="11">
-        <v>0</v>
-      </c>
-      <c r="L11" s="12">
+      <c r="K11" s="10">
+        <v>0</v>
+      </c>
+      <c r="L11" s="11">
         <v>0</v>
       </c>
       <c r="M11">
@@ -1693,42 +1690,42 @@
       <c r="P11">
         <v>0</v>
       </c>
-      <c r="Q11" s="11">
-        <v>0</v>
-      </c>
-      <c r="R11" s="12"/>
-      <c r="S11" s="20"/>
-      <c r="W11" s="11"/>
-      <c r="X11" s="12"/>
-      <c r="AC11" s="11"/>
+      <c r="Q11" s="10">
+        <v>0</v>
+      </c>
+      <c r="R11" s="11"/>
+      <c r="S11" s="17"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="11"/>
+      <c r="AC11" s="10"/>
       <c r="AD11" s="3">
-        <f>SUMPRODUCT(I11:AC11,$I$7:$AC$7)</f>
-        <v>239.99999999999994</v>
-      </c>
-      <c r="AE11" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF11" s="9">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="AE11" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="8">
         <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F12" s="8"/>
-      <c r="G12" s="13"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="33"/>
       <c r="H12" t="s">
         <v>2</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="11">
         <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="10">
         <f>1.1*20</f>
         <v>22</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <v>0</v>
       </c>
       <c r="M12">
@@ -1743,28 +1740,28 @@
       <c r="P12">
         <v>-1</v>
       </c>
-      <c r="Q12" s="11">
+      <c r="Q12" s="10">
         <v>-1</v>
       </c>
-      <c r="R12" s="12"/>
-      <c r="S12" s="20"/>
-      <c r="W12" s="11"/>
-      <c r="X12" s="12"/>
-      <c r="AC12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="17"/>
+      <c r="W12" s="10"/>
+      <c r="X12" s="11"/>
+      <c r="AC12" s="10"/>
       <c r="AD12" s="3">
-        <f>SUMPRODUCT(I12:AC12,$I$7:$AC$7)</f>
-        <v>0</v>
-      </c>
-      <c r="AE12" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF12" s="9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AE12" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F13" s="8"/>
-      <c r="G13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="5" t="s">
         <v>1</v>
       </c>
@@ -1808,92 +1805,92 @@
       <c r="AB13" s="5"/>
       <c r="AC13" s="4"/>
       <c r="AD13" s="3">
-        <f>SUMPRODUCT(I13:AC13,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>-5999.9999999999991</v>
       </c>
-      <c r="AE13" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF13" s="9">
+      <c r="AE13" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="8">
         <v>-6000</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F14" s="8"/>
-      <c r="G14" s="17" t="s">
+      <c r="F14" s="7"/>
+      <c r="G14" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="H14" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="14">
         <v>2.5</v>
       </c>
-      <c r="J14" s="15">
-        <v>0</v>
-      </c>
-      <c r="K14" s="14">
-        <v>0</v>
-      </c>
-      <c r="L14" s="16"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="16">
-        <v>1</v>
-      </c>
-      <c r="S14" s="15">
-        <v>0</v>
-      </c>
-      <c r="T14" s="15">
+      <c r="J14" s="13">
+        <v>0</v>
+      </c>
+      <c r="K14" s="12">
+        <v>0</v>
+      </c>
+      <c r="L14" s="14"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="14">
+        <v>1</v>
+      </c>
+      <c r="S14" s="13">
+        <v>0</v>
+      </c>
+      <c r="T14" s="13">
         <v>-1</v>
       </c>
-      <c r="U14" s="15">
-        <v>0</v>
-      </c>
-      <c r="V14" s="15">
-        <v>0</v>
-      </c>
-      <c r="W14" s="14">
-        <v>0</v>
-      </c>
-      <c r="X14" s="16"/>
-      <c r="Y14" s="15"/>
-      <c r="Z14" s="15"/>
-      <c r="AA14" s="15"/>
-      <c r="AB14" s="15"/>
-      <c r="AC14" s="14"/>
+      <c r="U14" s="13">
+        <v>0</v>
+      </c>
+      <c r="V14" s="13">
+        <v>0</v>
+      </c>
+      <c r="W14" s="12">
+        <v>0</v>
+      </c>
+      <c r="X14" s="14"/>
+      <c r="Y14" s="13"/>
+      <c r="Z14" s="13"/>
+      <c r="AA14" s="13"/>
+      <c r="AB14" s="13"/>
+      <c r="AC14" s="12"/>
       <c r="AD14" s="3">
-        <f>SUMPRODUCT(I14:AC14,$I$7:$AC$7)</f>
-        <v>200.00000000000026</v>
-      </c>
-      <c r="AE14" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="18">
+        <f t="shared" si="3"/>
+        <v>200.0000000000004</v>
+      </c>
+      <c r="AE14" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="15">
         <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F15" s="8"/>
-      <c r="G15" s="13"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="33"/>
       <c r="H15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="11">
         <v>0</v>
       </c>
       <c r="J15">
         <v>3</v>
       </c>
-      <c r="K15" s="11">
-        <v>0</v>
-      </c>
-      <c r="L15" s="12"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="12">
+      <c r="K15" s="10">
+        <v>0</v>
+      </c>
+      <c r="L15" s="11"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="11">
         <v>0</v>
       </c>
       <c r="S15">
@@ -1908,40 +1905,40 @@
       <c r="V15">
         <v>0</v>
       </c>
-      <c r="W15" s="11">
-        <v>0</v>
-      </c>
-      <c r="X15" s="12"/>
-      <c r="AC15" s="11"/>
+      <c r="W15" s="10">
+        <v>0</v>
+      </c>
+      <c r="X15" s="11"/>
+      <c r="AC15" s="10"/>
       <c r="AD15" s="3">
-        <f>SUMPRODUCT(I15:AC15,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>239.99999999999997</v>
       </c>
-      <c r="AE15" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF15" s="9">
+      <c r="AE15" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="8">
         <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="F16" s="8"/>
-      <c r="G16" s="13"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="33"/>
       <c r="H16" t="s">
         <v>2</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="11">
         <v>0</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="10">
         <v>20</v>
       </c>
-      <c r="L16" s="12"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="12">
+      <c r="L16" s="11"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="11">
         <v>0</v>
       </c>
       <c r="S16">
@@ -1956,25 +1953,25 @@
       <c r="V16">
         <v>-1</v>
       </c>
-      <c r="W16" s="11">
+      <c r="W16" s="10">
         <v>-1</v>
       </c>
-      <c r="X16" s="12"/>
-      <c r="AC16" s="11"/>
+      <c r="X16" s="11"/>
+      <c r="AC16" s="10"/>
       <c r="AD16" s="3">
-        <f>SUMPRODUCT(I16:AC16,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>-9.0949470177292824E-13</v>
       </c>
-      <c r="AE16" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF16" s="9">
+      <c r="AE16" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="6:32" x14ac:dyDescent="0.25">
-      <c r="F17" s="8"/>
-      <c r="G17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="34"/>
       <c r="H17" s="5" t="s">
         <v>1</v>
       </c>
@@ -2018,7 +2015,7 @@
       <c r="AB17" s="5"/>
       <c r="AC17" s="4"/>
       <c r="AD17" s="3">
-        <f>SUMPRODUCT(I17:AC17,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>-5454.545454545455</v>
       </c>
       <c r="AE17" s="2" t="s">
@@ -2029,85 +2026,85 @@
       </c>
     </row>
     <row r="18" spans="6:32" x14ac:dyDescent="0.25">
-      <c r="F18" s="8"/>
-      <c r="G18" s="17" t="s">
+      <c r="F18" s="7"/>
+      <c r="G18" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="14">
         <f>0.9*2.5</f>
         <v>2.25</v>
       </c>
-      <c r="J18" s="15">
-        <v>0</v>
-      </c>
-      <c r="K18" s="14">
-        <v>0</v>
-      </c>
-      <c r="L18" s="16"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="16"/>
-      <c r="S18" s="15"/>
-      <c r="T18" s="15"/>
-      <c r="U18" s="15"/>
-      <c r="V18" s="15"/>
-      <c r="W18" s="14"/>
-      <c r="X18" s="16">
-        <v>1</v>
-      </c>
-      <c r="Y18" s="15">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="15">
+      <c r="J18" s="13">
+        <v>0</v>
+      </c>
+      <c r="K18" s="12">
+        <v>0</v>
+      </c>
+      <c r="L18" s="14"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
+      <c r="V18" s="13"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="14">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="13">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="13">
         <v>-1</v>
       </c>
-      <c r="AA18" s="15">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="15">
-        <v>0</v>
-      </c>
-      <c r="AC18" s="14">
+      <c r="AA18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="12">
         <v>0</v>
       </c>
       <c r="AD18" s="3">
-        <f>SUMPRODUCT(I18:AC18,$I$7:$AC$7)</f>
-        <v>200.00000000000011</v>
-      </c>
-      <c r="AE18" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="9">
+        <f t="shared" si="3"/>
+        <v>200.00000000000017</v>
+      </c>
+      <c r="AE18" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="8">
         <v>200</v>
       </c>
     </row>
     <row r="19" spans="6:32" x14ac:dyDescent="0.25">
-      <c r="F19" s="8"/>
-      <c r="G19" s="13"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="33"/>
       <c r="H19" t="s">
         <v>3</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="11">
         <v>0</v>
       </c>
       <c r="J19">
         <f>0.9*3</f>
         <v>2.7</v>
       </c>
-      <c r="K19" s="11">
-        <v>0</v>
-      </c>
-      <c r="L19" s="12"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="12"/>
-      <c r="W19" s="11"/>
-      <c r="X19" s="12">
+      <c r="K19" s="10">
+        <v>0</v>
+      </c>
+      <c r="L19" s="11"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="11"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="11">
         <v>0</v>
       </c>
       <c r="Y19">
@@ -2122,41 +2119,41 @@
       <c r="AB19">
         <v>0</v>
       </c>
-      <c r="AC19" s="11">
+      <c r="AC19" s="10">
         <v>0</v>
       </c>
       <c r="AD19" s="3">
-        <f>SUMPRODUCT(I19:AC19,$I$7:$AC$7)</f>
-        <v>239.99999999999997</v>
-      </c>
-      <c r="AE19" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF19" s="9">
+        <f t="shared" si="3"/>
+        <v>240</v>
+      </c>
+      <c r="AE19" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="8">
         <v>240</v>
       </c>
     </row>
     <row r="20" spans="6:32" x14ac:dyDescent="0.25">
-      <c r="F20" s="8"/>
-      <c r="G20" s="13"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="33"/>
       <c r="H20" t="s">
         <v>2</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
         <v>0</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20" s="10">
         <f>0.9*20</f>
         <v>18</v>
       </c>
-      <c r="L20" s="12"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="12"/>
-      <c r="W20" s="11"/>
-      <c r="X20" s="12">
+      <c r="L20" s="11"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="11"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="11">
         <v>0</v>
       </c>
       <c r="Y20">
@@ -2171,23 +2168,23 @@
       <c r="AB20">
         <v>-1</v>
       </c>
-      <c r="AC20" s="11">
+      <c r="AC20" s="10">
         <v>-1</v>
       </c>
       <c r="AD20" s="3">
-        <f>SUMPRODUCT(I20:AC20,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>-9.0949470177292824E-13</v>
       </c>
-      <c r="AE20" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="9">
+      <c r="AE20" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="6:32" x14ac:dyDescent="0.25">
-      <c r="F21" s="8"/>
-      <c r="G21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="34"/>
       <c r="H21" s="5" t="s">
         <v>1</v>
       </c>
@@ -2231,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AD21" s="3">
-        <f>SUMPRODUCT(I21:AC21,$I$7:$AC$7)</f>
+        <f t="shared" si="3"/>
         <v>-4909.090909090909</v>
       </c>
       <c r="AE21" s="2" t="s">

</xml_diff>